<commit_message>
Update HYPE and MEME trading lessons
</commit_message>
<xml_diff>
--- a/workspace/trade_journal.xlsx
+++ b/workspace/trade_journal.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="统计" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'合约复盘'!$A$1:$R$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'合约复盘'!$A$1:$R$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:R15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1757,8 +1757,100 @@
         </is>
       </c>
     </row>
+    <row r="15" ht="86" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>T014</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-31 20:57:05</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-31 22:02:36</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>1000PEPEUSDT</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>做多</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>2900</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>0.0034415</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>0.0034190</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>0.003420</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>失败止损</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>-0.06525000</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>0.00994771</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>-0.07519771</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>2x杠杆 约9.98U名义仓位 约4.99U保证金 小仓meme试单止损退出</t>
+        </is>
+      </c>
+      <c r="O15" s="5" t="inlineStr">
+        <is>
+          <t>5/10</t>
+        </is>
+      </c>
+      <c r="P15" s="4" t="inlineStr">
+        <is>
+          <t>1000PEPE作为当时meme候选龙一 15m/1h结构较强 但入场后没有站稳0.003445 反而回落触发保护止损</t>
+        </is>
+      </c>
+      <c r="Q15" s="4" t="inlineStr">
+        <is>
+          <t>失败原因是突破确认不够扎实 多头账户拥挤且taker卖压切换明显 入场后未能快速打到第一目标 说明这笔属于试单失败而非策略大错</t>
+        </is>
+      </c>
+      <c r="R15" s="4" t="inlineStr">
+        <is>
+          <t>热点meme小试可以做 但已有卖压警告时必须等0.003445真正站稳或回踩确认；止损后不立刻追回 除非重新站回关键位并形成新结构</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R14"/>
+  <autoFilter ref="A1:R15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1795,7 +1887,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -1815,7 +1907,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
@@ -1826,7 +1918,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>23.1%</t>
+          <t>21.4%</t>
         </is>
       </c>
     </row>
@@ -1837,7 +1929,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.554566</v>
+        <v>-0.629763</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record MEME stop-out lesson
</commit_message>
<xml_diff>
--- a/workspace/trade_journal.xlsx
+++ b/workspace/trade_journal.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="统计" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'合约复盘'!$A$1:$R$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'合约复盘'!$A$1:$R$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R15"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1849,8 +1849,100 @@
         </is>
       </c>
     </row>
+    <row r="16" ht="86" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>T015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01 10:15:35</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01 10:22:23</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>MEMEUSDT</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>做多</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>8000</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>0.0006331</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>0.0006115</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>0.000612</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>失败止损</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>-0.17280000</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>0.00497839</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>-0.17777839</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>half-size momentum test loss; stopped by normal pullback after late chase</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>MEME方向强但入场太急，追在0.000630突破后的强拉末端，未等待0.000625回踩确认；BTC仍偏弱且多头拥挤，止损位被正常回抽打掉。</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>失败原因是节奏过急：把1m/5m冲高当成确认，没有等突破后回踩站稳；入场后仅7分钟触发止损，说明位置处在洗盘/回抽区。</t>
+        </is>
+      </c>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>所有强势币和meme通用：追涨后必须有二次确认；强拉末端只允许更小试单或不做；若BTC弱且多头拥挤，优先等回踩0.000625附近站稳或新结构，不在突破高位直接补票。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R15"/>
+  <autoFilter ref="A1:R16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1887,7 +1979,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -1907,7 +1999,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -1918,7 +2010,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>21.4%</t>
+          <t>20.0%</t>
         </is>
       </c>
     </row>
@@ -1929,7 +2021,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.629763</v>
+        <v>-0.807542</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record HYPE stop-out review
</commit_message>
<xml_diff>
--- a/workspace/trade_journal.xlsx
+++ b/workspace/trade_journal.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="统计" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'合约复盘'!$A$1:$R$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'合约复盘'!$A$1:$R$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R16"/>
+  <dimension ref="A1:R17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1941,8 +1941,100 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="86" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>T016</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01 11:16:02</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01 11:29:31</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>HYPEUSDT</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>做多</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>0.13</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>72.916</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>72.372</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>72.38</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>失败止损</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>-0.07072000</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>0.00944372</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>-0.08016372</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>small test loss; stop slipped slightly below trigger</t>
+        </is>
+      </c>
+      <c r="O17" s="5" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="P17" s="4" t="inlineStr">
+        <is>
+          <t>HYPE方向仍是强势主线，但这笔追在冲高后的二次反弹，回踩确认不够厚；72.38止损低于短线回踩位但仍处在HYPE快速洗盘范围内。</t>
+        </is>
+      </c>
+      <c r="Q17" s="4" t="inlineStr">
+        <is>
+          <t>失败原因是上车点仍偏高，73.128冲高后虽然回踩72.68守住，但没有等更充分的5m结构确认；后续回落打穿72.38，说明该段反弹承接不足。</t>
+        </is>
+      </c>
+      <c r="R17" s="4" t="inlineStr">
+        <is>
+          <t>HYPE强势币继续允许做多，但下一次必须等更深回踩或二次站稳：优先等接近15m EMA9/关键结构位承接，或突破73.13后回踩不破；刚被止损后不立刻同方向追，除非形成新结构。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R16"/>
+  <autoFilter ref="A1:R17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1979,7 +2071,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
@@ -1999,7 +2091,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
@@ -2010,7 +2102,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>18.8%</t>
         </is>
       </c>
     </row>
@@ -2021,7 +2113,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.807542</v>
+        <v>-0.887706</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record HYPE repair-zone stop-out
</commit_message>
<xml_diff>
--- a/workspace/trade_journal.xlsx
+++ b/workspace/trade_journal.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="统计" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'合约复盘'!$A$1:$R$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'合约复盘'!$A$1:$R$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R17"/>
+  <dimension ref="A1:R18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2033,8 +2033,100 @@
         </is>
       </c>
     </row>
+    <row r="18" ht="86" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>T017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01 16:11:12</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01 16:36:54</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>HYPEUSDT</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>做多</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>0.13</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>72.799</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>72.180</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>72.28</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>失败止损</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>-0.08047000</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>0.00942363</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>-0.08989363</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>small test loss; BTC strong-down invalidated repair attempt</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>HYPE本身仍相对强，但BTC持续强空，HYPE 5m/15m没有完成转强，只是修复区反抽；入场后未能站稳72.90-73.00，随后被大盘拖回并触发止损。</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>失败原因是把修复区反抽当成可试多机会，BTC 1m/5m/15m/1h/4h偏空时，HYPE需要更高确认；72.28虽低于短线结构，但仍挡不住大盘下杀。</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>BTC三周期强空时，HYPE修复区多单必须降级：只有站稳15m EMA21上方并5m转强，或深回踩到15m/1h结构位出现放量承接，才允许试；否则不因taker短暂转买就开多。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R17"/>
+  <autoFilter ref="A1:R18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2071,7 +2163,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -2091,7 +2183,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
@@ -2102,7 +2194,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>18.8%</t>
+          <t>17.6%</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2205,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.887706</v>
+        <v>-0.977599</v>
       </c>
     </row>
   </sheetData>

</xml_diff>